<commit_message>
Register: D89 foreloebig slettefrist (3 mdr / 12 mdr gensalg), D91 gentilmelding uden login-kobling
</commit_message>
<xml_diff>
--- a/docs/databehandleraftaler/gdpr.xlsx
+++ b/docs/databehandleraftaler/gdpr.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\sms-backend\docs\databehandleraftaler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F50D8E-EA3F-4C77-A8C0-FD031CF502C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C04CC2-FE79-421A-8CFD-8881237BCF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="137">
   <si>
     <t>Dit Digitale Kontor - GDPR Master</t>
   </si>
@@ -431,6 +431,15 @@
   </si>
   <si>
     <t>lytte, læse skriv referater pba talt tekst og referater</t>
+  </si>
+  <si>
+    <t>navn, firmannavn, mail og telefonnummer opbevares et år</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alle andre kundedata, og kundens kundedata slette efter 3 måneder </t>
+  </si>
+  <si>
+    <t>denne bruges til gensalg,</t>
   </si>
 </sst>
 </file>
@@ -1428,15 +1437,28 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>62</v>
       </c>
       <c r="B1" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>